<commit_message>
whore(doc): adiciona tabelas atualizadas
</commit_message>
<xml_diff>
--- a/Tabelas/casos_por_ano.xlsx
+++ b/Tabelas/casos_por_ano.xlsx
@@ -458,7 +458,7 @@
         <v>1875</v>
       </c>
       <c r="D2" t="n">
-        <v>32.3</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         <v>1260</v>
       </c>
       <c r="D3" t="n">
-        <v>21.71</v>
+        <v>20.49</v>
       </c>
     </row>
     <row r="4">
@@ -490,7 +490,7 @@
         <v>682</v>
       </c>
       <c r="D4" t="n">
-        <v>11.75</v>
+        <v>11.09</v>
       </c>
     </row>
     <row r="5">
@@ -506,7 +506,7 @@
         <v>667</v>
       </c>
       <c r="D5" t="n">
-        <v>11.49</v>
+        <v>10.85</v>
       </c>
     </row>
     <row r="6">
@@ -522,7 +522,7 @@
         <v>541</v>
       </c>
       <c r="D6" t="n">
-        <v>9.32</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -538,7 +538,7 @@
         <v>522</v>
       </c>
       <c r="D7" t="n">
-        <v>8.99</v>
+        <v>8.49</v>
       </c>
     </row>
     <row r="8">
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>258</v>
+        <v>601</v>
       </c>
       <c r="D8" t="n">
-        <v>4.44</v>
+        <v>9.779999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>